<commit_message>
HO6 DONE,recording the information of your favorite people using python and creating excel file to store the data
</commit_message>
<xml_diff>
--- a/HO6_fav_people/favorite_people.xlsx
+++ b/HO6_fav_people/favorite_people.xlsx
@@ -449,19 +449,19 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Oswald</t>
+          <t>Andrei</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Pastorfide</t>
+          <t>Menemedez</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>2004</v>
+        <v>2005</v>
       </c>
       <c r="E2" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="3">
@@ -470,19 +470,19 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Jdadawdaw</t>
+          <t>Oswald</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>dwadawdaw</t>
+          <t>Pastorfide</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>2000</v>
+        <v>2003</v>
       </c>
       <c r="E3" t="n">
-        <v>26</v>
+        <v>23</v>
       </c>
     </row>
     <row r="4">
@@ -491,12 +491,12 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>dawdada</t>
+          <t>jeph</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>awdawda</t>
+          <t>Dellosa</t>
         </is>
       </c>
       <c r="D4" t="n">

</xml_diff>